<commit_message>
Merged PR 2489: Merge planningmodulenewscenarios to master
</commit_message>
<xml_diff>
--- a/src/main/resources/SiteVisit_Field_Values.xlsx
+++ b/src/main/resources/SiteVisit_Field_Values.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E54552E-2C3E-4371-A6C0-EDFA2B456CC9}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E13C3A-C5C7-434B-8B16-2647E968F0AB}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
-    <sheet name="Outcomes" sheetId="6" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="7" r:id="rId4"/>
-    <sheet name="Edition" sheetId="3" r:id="rId5"/>
-    <sheet name="Form Fields1" sheetId="5" r:id="rId6"/>
-    <sheet name="Form Fields" sheetId="8" r:id="rId7"/>
+    <sheet name="Creation1" sheetId="10" r:id="rId2"/>
+    <sheet name="Outcomes" sheetId="6" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId5"/>
+    <sheet name="Edition" sheetId="3" r:id="rId6"/>
+    <sheet name="Sheet3" sheetId="9" r:id="rId7"/>
+    <sheet name="Form Fields1" sheetId="5" r:id="rId8"/>
+    <sheet name="Form Fields" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="109">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -355,6 +357,9 @@
   </si>
   <si>
     <t>fieldSupportingCommentsQuestion1__c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Program </t>
   </si>
 </sst>
 </file>
@@ -727,13 +732,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -744,7 +749,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -755,7 +760,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -766,7 +771,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -783,16 +788,74 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1F38FE0-E02C-4583-8E5B-5FC537096D3A}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79F1E74-3E81-4D35-A66E-768A31821CE0}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -803,7 +866,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>28</v>
       </c>
@@ -814,7 +877,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>28</v>
       </c>
@@ -825,7 +888,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>28</v>
       </c>
@@ -836,7 +899,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>28</v>
       </c>
@@ -853,15 +916,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -869,7 +932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -877,7 +940,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -885,7 +948,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -893,67 +956,24 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>22</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2233F5ED-8740-43F6-9895-B674ACB6DEF9}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -962,16 +982,59 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2233F5ED-8740-43F6-9895-B674ACB6DEF9}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -982,7 +1045,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -993,7 +1056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1004,7 +1067,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1015,7 +1078,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1026,7 +1089,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1037,7 +1100,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1048,7 +1111,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1065,16 +1128,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4D4A9-3A34-4259-AC25-4E874229397A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F8298A-0165-44BF-9061-10BEE0A93A27}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="106.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1085,7 +1157,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1096,7 +1168,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1107,7 +1179,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1118,7 +1190,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1129,7 +1201,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1140,7 +1212,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1151,7 +1223,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1162,7 +1234,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1173,7 +1245,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1184,7 +1256,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1195,7 +1267,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1206,7 +1278,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1217,7 +1289,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1228,7 +1300,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1239,7 +1311,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1250,7 +1322,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1261,7 +1333,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1272,7 +1344,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1283,7 +1355,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1294,7 +1366,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1305,7 +1377,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1316,7 +1388,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1327,7 +1399,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1338,7 +1410,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1349,7 +1421,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1360,7 +1432,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1371,7 +1443,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1382,7 +1454,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1393,7 +1465,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1409,17 +1481,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC98D198-04E6-490A-B46B-512D2A0BE3E3}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1430,7 +1502,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1441,7 +1513,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1452,7 +1524,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1463,7 +1535,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1474,7 +1546,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1485,7 +1557,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1496,7 +1568,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -1507,7 +1579,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1518,7 +1590,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -1529,7 +1601,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B13" s="4"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated test cases for award #1
</commit_message>
<xml_diff>
--- a/src/main/resources/SiteVisit_Field_Values.xlsx
+++ b/src/main/resources/SiteVisit_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29FBC96-C4B5-4E0C-B4F6-616562DA181F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D06C5EB3-710E-412F-A2EE-5904F7D80344}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="10" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="1" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -118,9 +118,6 @@
     <t>SvProgramFormQ4__c</t>
   </si>
   <si>
-    <t xml:space="preserve">Automation Site Visit </t>
-  </si>
-  <si>
     <t>Reports and Outcomes</t>
   </si>
   <si>
@@ -362,6 +359,9 @@
   </si>
   <si>
     <t xml:space="preserve">Program </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Runtime Site Visit </t>
   </si>
 </sst>
 </file>
@@ -734,13 +734,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -751,7 +751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -759,10 +759,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -773,7 +773,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -792,13 +792,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F8298A-0165-44BF-9061-10BEE0A93A27}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="106.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -809,271 +809,271 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>38</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>42</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>44</v>
       </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>50</v>
       </c>
-      <c r="C9" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>52</v>
       </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>54</v>
       </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>56</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>58</v>
       </c>
-      <c r="C13" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>60</v>
       </c>
-      <c r="C14" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>62</v>
       </c>
-      <c r="C15" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>64</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>66</v>
       </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>68</v>
       </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>70</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>72</v>
       </c>
-      <c r="C20" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>74</v>
       </c>
-      <c r="C21" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>76</v>
       </c>
-      <c r="C22" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>78</v>
       </c>
-      <c r="C23" t="s">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>80</v>
       </c>
-      <c r="C24" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>4</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>82</v>
       </c>
-      <c r="C25" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1081,10 +1081,10 @@
         <v>23</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1092,10 +1092,10 @@
         <v>24</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1103,10 +1103,10 @@
         <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1114,18 +1114,18 @@
         <v>26</v>
       </c>
       <c r="C29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>4</v>
-      </c>
-      <c r="B30" t="s">
-        <v>88</v>
-      </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1136,14 +1136,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC98D198-04E6-490A-B46B-512D2A0BE3E3}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1162,10 +1162,10 @@
         <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1173,10 +1173,10 @@
         <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1184,10 +1184,10 @@
         <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1195,65 +1195,65 @@
         <v>26</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="1" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="1" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C9" s="1" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="B13" s="4"/>
     </row>
   </sheetData>
@@ -1265,13 +1265,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1F38FE0-E02C-4583-8E5B-5FC537096D3A}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1290,10 +1290,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1323,14 +1323,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79F1E74-3E81-4D35-A66E-768A31821CE0}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1341,48 +1341,48 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" t="s">
         <v>30</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" t="s">
         <v>32</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" t="s">
         <v>34</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1394,12 +1394,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1431,22 +1431,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B8" t="s">
         <v>22</v>
       </c>
@@ -1459,39 +1459,39 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2233F5ED-8740-43F6-9895-B674ACB6DEF9}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
         <v>30</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" t="s">
         <v>34</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1502,14 +1502,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1531,7 +1531,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1542,56 +1542,56 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
         <v>18</v>
@@ -1606,13 +1606,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939E4119-ACED-4858-8093-FD1B7FF9F1D3}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1645,45 +1645,45 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
@@ -1697,13 +1697,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E614565-35C2-477C-A727-DE66F54E56C3}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1736,45 +1736,45 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
@@ -1788,7 +1788,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F4D4A9-3A34-4259-AC25-4E874229397A}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Removed Duplicate steps from local
</commit_message>
<xml_diff>
--- a/src/main/resources/SiteVisit_Field_Values.xlsx
+++ b/src/main/resources/SiteVisit_Field_Values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05363EE0-E4DA-4D56-84E8-D3619DE019EB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADAC9E5B-DE94-4427-A943-67A3EE0F91AE}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
@@ -1285,7 +1285,7 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="20.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">

</xml_diff>